<commit_message>
#43 Added pull-up resistor and cap on EN pin, BOM and deliverables generated
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.5/BOM/Client-BOM-IoT-Button-v1.5.xlsx
+++ b/Design Files/IoT-Button-v1.5/BOM/Client-BOM-IoT-Button-v1.5.xlsx
@@ -80,7 +80,7 @@
     <t>1uF</t>
   </si>
   <si>
-    <t>C5, C8, C10, C11, C12, C14, C15, C16, C17, C18, C22, C23</t>
+    <t>C2, C5, C8, C10, C11, C12, C14, C15, C16, C17, C18, C22, C23</t>
   </si>
   <si>
     <t>CAP CER 0.1UF 25V X5R 0402</t>
@@ -113,6 +113,9 @@
     <t>Nexperia</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>Fuse</t>
   </si>
   <si>
@@ -215,13 +218,10 @@
     <t>TECH PUBLIC</t>
   </si>
   <si>
-    <t>Si2302CDS</t>
-  </si>
-  <si>
     <t>Resistor</t>
   </si>
   <si>
-    <t>R6, R9, R10, R13, R14</t>
+    <t>R1, R6, R9, R10, R13, R14</t>
   </si>
   <si>
     <t>RES SMD 10K Ohm 1% 1/10W 0603</t>
@@ -1538,11 +1538,11 @@
         <v>21</v>
       </c>
       <c r="J4" s="12">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" ht="15.75" spans="1:11">
+    <row r="5" spans="1:11">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
         <f>ROW(B5)-ROW($B$2)</f>
@@ -1567,7 +1567,7 @@
         <v>27</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J5" s="9">
         <v>1</v>
@@ -1581,57 +1581,57 @@
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>32</v>
       </c>
       <c r="J6" s="12">
         <v>1</v>
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="15.75" spans="1:11">
+    <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f>ROW(B7)-ROW($B$2)</f>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="J7" s="9">
         <v>1</v>
@@ -1645,25 +1645,25 @@
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="I8" s="13" t="s">
-        <v>43</v>
+        <v>45</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="J8" s="12">
         <v>1</v>
@@ -1677,25 +1677,25 @@
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="J9" s="9">
         <v>1</v>
@@ -1709,64 +1709,64 @@
         <v>8</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="I10" s="13" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="J10" s="12">
         <v>6</v>
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" ht="15.75" spans="1:11">
+    <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
         <f>ROW(B11)-ROW($B$2)</f>
         <v>9</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="J11" s="9">
         <v>1</v>
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" ht="15.75" spans="1:11">
+    <row r="12" spans="1:11">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
         <f>ROW(B12)-ROW($B$2)</f>
@@ -1794,11 +1794,11 @@
         <v>68</v>
       </c>
       <c r="J12" s="12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K12" s="12"/>
     </row>
-    <row r="13" ht="15.75" spans="1:11">
+    <row r="13" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
         <f>ROW(B13)-ROW($B$2)</f>
@@ -1855,7 +1855,7 @@
         <v>77</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="J14" s="12">
         <v>1</v>
@@ -1886,15 +1886,15 @@
       <c r="H15" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="I15" s="10" t="s">
-        <v>80</v>
+      <c r="I15" s="13" t="s">
+        <v>28</v>
       </c>
       <c r="J15" s="9">
         <v>1</v>
       </c>
       <c r="K15" s="9"/>
     </row>
-    <row r="16" ht="24.75" spans="1:11">
+    <row r="16" spans="1:11">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
         <f>ROW(B16)-ROW($B$2)</f>
@@ -1919,14 +1919,14 @@
         <v>87</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>86</v>
+        <v>28</v>
       </c>
       <c r="J16" s="12">
         <v>1</v>
       </c>
       <c r="K16" s="12"/>
     </row>
-    <row r="17" ht="15.75" spans="1:11">
+    <row r="17" spans="1:11">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
         <f>ROW(B17)-ROW($B$2)</f>
@@ -1950,8 +1950,8 @@
       <c r="H17" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="I17" s="10" t="s">
-        <v>92</v>
+      <c r="I17" s="13" t="s">
+        <v>28</v>
       </c>
       <c r="J17" s="9">
         <v>1</v>

</xml_diff>